<commit_message>
Add new reference ground truth: LAEC/CSE Tier 1, TAD Filing, AUS/NZ FAK/Tier 1, LAEC LUX, EAF-TZDAR OPUS
New MRG+OPUS pairs for several lane families identified in the latest
reference/ scan: LAEC FAK/Tier 1 extra weeks, CSE Tier 1, TAD Filing (all
3 variants' first week), AUS SEA to AUBP FAK/Tier 1, AUS NEA to AUEC
FAK, NZ1/NZJ FAK, LAEC LUX, and EAF-TZDAR's first real OPUS ground
truth. Also adds the TAD filing tooling (Tool for TAD.xlsm + its VBA
export module) and a surcharge code/definition reference sheet, plus an
updated hackathon tracker.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/for hackathon TRACKER.xlsx
+++ b/reference/for hackathon TRACKER.xlsx
@@ -5,13 +5,15 @@
   <sheets>
     <sheet state="visible" name="Sheet2" sheetId="1" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Sheet2!$A$1:$H$114</definedName>
+  </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="48">
   <si>
     <t>No.</t>
   </si>
@@ -58,9 +60,6 @@
     <t>INPUT: CSE TIER 1, CSE TIER 1 FOR VELAG AND VEPBL</t>
   </si>
   <si>
-    <t>In progress</t>
-  </si>
-  <si>
     <t>INPUT: EAF-TZDAR</t>
   </si>
   <si>
@@ -85,6 +84,9 @@
     <t>INPUT: West Asia to WAF_SAF_EAF_MZ</t>
   </si>
   <si>
+    <t>Ralfjhon Barbuena</t>
+  </si>
+  <si>
     <t>Not started</t>
   </si>
   <si>
@@ -95,9 +97,6 @@
   </si>
   <si>
     <t>INPUT: LAEC FAK</t>
-  </si>
-  <si>
-    <t>Ralfjhon Barbuena</t>
   </si>
   <si>
     <t>OUTPUT: OPUS RATES, CMDT NOTE, ROUTE NOTE, ORIGIN ARBS, SPECIAL NOTE</t>
@@ -187,6 +186,11 @@
     </font>
     <font>
       <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
       <color rgb="FF434343"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -194,11 +198,6 @@
     <font>
       <u/>
       <color rgb="FF434343"/>
-      <name val="Roboto"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
       <name val="Roboto"/>
     </font>
     <font>
@@ -266,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -297,12 +296,6 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -310,7 +303,16 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -404,6 +406,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H114" displayName="Project_tasks" name="Project_tasks" id="1">
+  <autoFilter ref="$A$1:$H$114"/>
   <tableColumns count="8">
     <tableColumn name="No." id="1"/>
     <tableColumn name="Task" id="2"/>
@@ -756,14 +759,20 @@
         <v>14</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
+      <c r="E6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G6" s="7">
+        <v>46255.0</v>
+      </c>
       <c r="H6" s="8"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -774,14 +783,20 @@
         <v>12</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
+      <c r="E7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G7" s="7">
+        <v>46255.0</v>
+      </c>
       <c r="H7" s="8"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
@@ -792,14 +807,20 @@
         <v>14</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
+      <c r="E8" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="7">
+        <v>46256.0</v>
+      </c>
+      <c r="G8" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H8" s="8"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
@@ -810,14 +831,20 @@
         <v>12</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
+      <c r="E9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="7">
+        <v>46256.0</v>
+      </c>
+      <c r="G9" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H9" s="8"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
@@ -825,17 +852,23 @@
         <v>5.0</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
+      <c r="E10" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="7">
+        <v>46253.0</v>
+      </c>
+      <c r="G10" s="7">
+        <v>46259.0</v>
+      </c>
       <c r="H10" s="8"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
@@ -843,17 +876,23 @@
         <v>5.0</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
+      <c r="E11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="7">
+        <v>46253.0</v>
+      </c>
+      <c r="G11" s="7">
+        <v>46259.0</v>
+      </c>
       <c r="H11" s="8"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
@@ -861,17 +900,23 @@
         <v>6.0</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
+      <c r="E12" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="7">
+        <v>46260.0</v>
+      </c>
+      <c r="G12" s="7">
+        <v>46266.0</v>
+      </c>
       <c r="H12" s="8"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
@@ -879,17 +924,23 @@
         <v>6.0</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
+      <c r="E13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="7">
+        <v>46260.0</v>
+      </c>
+      <c r="G13" s="7">
+        <v>46266.0</v>
+      </c>
       <c r="H13" s="8"/>
     </row>
     <row r="14" ht="22.5" customHeight="1">
@@ -897,7 +948,7 @@
         <v>7.0</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>9</v>
@@ -905,7 +956,7 @@
       <c r="D14" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="7">
@@ -921,7 +972,7 @@
         <v>7.0</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>9</v>
@@ -945,7 +996,7 @@
         <v>8.0</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>9</v>
@@ -953,7 +1004,7 @@
       <c r="D16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="7">
@@ -969,7 +1020,7 @@
         <v>8.0</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>9</v>
@@ -993,15 +1044,15 @@
         <v>9.0</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="11" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="7">
@@ -1017,15 +1068,15 @@
         <v>9.0</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E19" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="7">
@@ -1041,15 +1092,15 @@
         <v>10.0</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E20" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="7">
@@ -1065,15 +1116,15 @@
         <v>10.0</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F21" s="7">
@@ -1089,22 +1140,22 @@
         <v>11.0</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E22" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F22" s="7">
         <v>46235.0</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H22" s="8"/>
     </row>
@@ -1113,22 +1164,22 @@
         <v>11.0</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E23" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F23" s="7">
         <v>46235.0</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H23" s="8"/>
     </row>
@@ -1137,15 +1188,15 @@
         <v>12.0</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E24" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F24" s="7">
@@ -1161,15 +1212,15 @@
         <v>12.0</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F25" s="7">
@@ -1185,17 +1236,21 @@
         <v>13.0</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C26" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E26" s="10"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G26" s="7">
+        <v>46279.0</v>
+      </c>
       <c r="H26" s="8"/>
     </row>
     <row r="27" ht="22.5" customHeight="1">
@@ -1203,17 +1258,15 @@
         <v>13.0</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27" s="10"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
       <c r="H27" s="8"/>
     </row>
     <row r="28" ht="22.5" customHeight="1">
@@ -1221,17 +1274,21 @@
         <v>14.0</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C28" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E28" s="10"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G28" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H28" s="8"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
@@ -1239,17 +1296,15 @@
         <v>14.0</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E29" s="10"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
       <c r="H29" s="8"/>
     </row>
     <row r="30" ht="22.5" customHeight="1">
@@ -1263,9 +1318,9 @@
         <v>9</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E30" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E30" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F30" s="7">
@@ -1281,15 +1336,15 @@
         <v>15.0</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E31" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F31" s="7">
@@ -1311,9 +1366,9 @@
         <v>9</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E32" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="7">
@@ -1329,15 +1384,15 @@
         <v>16.0</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E33" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F33" s="7">
@@ -1359,9 +1414,9 @@
         <v>9</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E34" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F34" s="7">
@@ -1377,15 +1432,15 @@
         <v>17.0</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E35" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F35" s="7">
@@ -1407,9 +1462,9 @@
         <v>9</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E36" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="7">
@@ -1425,15 +1480,15 @@
         <v>18.0</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E37" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F37" s="7">
@@ -1455,11 +1510,9 @@
         <v>9</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E38" s="13" t="s">
-        <v>11</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="E38" s="15"/>
       <c r="F38" s="7">
         <v>46266.0</v>
       </c>
@@ -1473,17 +1526,15 @@
         <v>19.0</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>13</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="E39" s="15"/>
       <c r="F39" s="7">
         <v>46266.0</v>
       </c>
@@ -1500,14 +1551,18 @@
         <v>27</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E40" s="10"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E40" s="12"/>
+      <c r="F40" s="7">
+        <v>46256.0</v>
+      </c>
+      <c r="G40" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H40" s="8"/>
     </row>
     <row r="41" ht="22.5" customHeight="1">
@@ -1515,17 +1570,21 @@
         <v>20.0</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E41" s="10"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E41" s="12"/>
+      <c r="F41" s="7">
+        <v>46256.0</v>
+      </c>
+      <c r="G41" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H41" s="8"/>
     </row>
     <row r="42" ht="22.5" customHeight="1">
@@ -1533,17 +1592,21 @@
         <v>21.0</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E42" s="10"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E42" s="12"/>
+      <c r="F42" s="7">
+        <v>46256.0</v>
+      </c>
+      <c r="G42" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H42" s="8"/>
     </row>
     <row r="43" ht="22.5" customHeight="1">
@@ -1551,17 +1614,21 @@
         <v>21.0</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E43" s="10"/>
-      <c r="F43" s="11"/>
-      <c r="G43" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E43" s="12"/>
+      <c r="F43" s="7">
+        <v>46256.0</v>
+      </c>
+      <c r="G43" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H43" s="8"/>
     </row>
     <row r="44" ht="22.5" customHeight="1">
@@ -1569,17 +1636,21 @@
         <v>22.0</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E44" s="10"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E44" s="12"/>
+      <c r="F44" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G44" s="7">
+        <v>46272.0</v>
+      </c>
       <c r="H44" s="8"/>
     </row>
     <row r="45" ht="22.5" customHeight="1">
@@ -1587,17 +1658,21 @@
         <v>22.0</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E45" s="10"/>
-      <c r="F45" s="11"/>
-      <c r="G45" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E45" s="12"/>
+      <c r="F45" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G45" s="7">
+        <v>46272.0</v>
+      </c>
       <c r="H45" s="8"/>
     </row>
     <row r="46" ht="22.5" customHeight="1">
@@ -1605,17 +1680,17 @@
         <v>23.0</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E46" s="10"/>
-      <c r="F46" s="11"/>
-      <c r="G46" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E46" s="12"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="14"/>
       <c r="H46" s="8"/>
     </row>
     <row r="47" ht="22.5" customHeight="1">
@@ -1623,17 +1698,17 @@
         <v>23.0</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E47" s="10"/>
-      <c r="F47" s="11"/>
-      <c r="G47" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E47" s="12"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="14"/>
       <c r="H47" s="8"/>
     </row>
     <row r="48" ht="22.5" customHeight="1">
@@ -1641,17 +1716,17 @@
         <v>24.0</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E48" s="10"/>
-      <c r="F48" s="11"/>
-      <c r="G48" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E48" s="12"/>
+      <c r="F48" s="14"/>
+      <c r="G48" s="14"/>
       <c r="H48" s="8"/>
     </row>
     <row r="49" ht="22.5" customHeight="1">
@@ -1659,17 +1734,17 @@
         <v>24.0</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E49" s="10"/>
-      <c r="F49" s="11"/>
-      <c r="G49" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E49" s="12"/>
+      <c r="F49" s="14"/>
+      <c r="G49" s="14"/>
       <c r="H49" s="8"/>
     </row>
     <row r="50" ht="22.5" customHeight="1">
@@ -1677,17 +1752,17 @@
         <v>25.0</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E50" s="10"/>
-      <c r="F50" s="11"/>
-      <c r="G50" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E50" s="12"/>
+      <c r="F50" s="14"/>
+      <c r="G50" s="14"/>
       <c r="H50" s="8"/>
     </row>
     <row r="51" ht="22.5" customHeight="1">
@@ -1695,17 +1770,17 @@
         <v>25.0</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E51" s="10"/>
-      <c r="F51" s="11"/>
-      <c r="G51" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E51" s="12"/>
+      <c r="F51" s="14"/>
+      <c r="G51" s="14"/>
       <c r="H51" s="8"/>
     </row>
     <row r="52" ht="22.5" customHeight="1">
@@ -1713,17 +1788,17 @@
         <v>26.0</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E52" s="10"/>
-      <c r="F52" s="11"/>
-      <c r="G52" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E52" s="12"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
       <c r="H52" s="8"/>
     </row>
     <row r="53" ht="22.5" customHeight="1">
@@ -1731,17 +1806,17 @@
         <v>26.0</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E53" s="10"/>
-      <c r="F53" s="11"/>
-      <c r="G53" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E53" s="12"/>
+      <c r="F53" s="14"/>
+      <c r="G53" s="14"/>
       <c r="H53" s="8"/>
     </row>
     <row r="54" ht="22.5" customHeight="1">
@@ -1749,17 +1824,17 @@
         <v>27.0</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E54" s="10"/>
-      <c r="F54" s="11"/>
-      <c r="G54" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E54" s="12"/>
+      <c r="F54" s="14"/>
+      <c r="G54" s="14"/>
       <c r="H54" s="8"/>
     </row>
     <row r="55" ht="22.5" customHeight="1">
@@ -1767,17 +1842,17 @@
         <v>27.0</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E55" s="10"/>
-      <c r="F55" s="11"/>
-      <c r="G55" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E55" s="12"/>
+      <c r="F55" s="14"/>
+      <c r="G55" s="14"/>
       <c r="H55" s="8"/>
     </row>
     <row r="56" ht="22.5" customHeight="1">
@@ -1785,17 +1860,17 @@
         <v>28.0</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E56" s="10"/>
-      <c r="F56" s="11"/>
-      <c r="G56" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E56" s="12"/>
+      <c r="F56" s="14"/>
+      <c r="G56" s="14"/>
       <c r="H56" s="8"/>
     </row>
     <row r="57" ht="22.5" customHeight="1">
@@ -1803,17 +1878,17 @@
         <v>28.0</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E57" s="10"/>
-      <c r="F57" s="11"/>
-      <c r="G57" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="E57" s="12"/>
+      <c r="F57" s="14"/>
+      <c r="G57" s="14"/>
       <c r="H57" s="8"/>
     </row>
     <row r="58" ht="22.5" customHeight="1">
@@ -1821,15 +1896,15 @@
         <v>29.0</v>
       </c>
       <c r="B58" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C58" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D58" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E58" s="13" t="s">
+      <c r="E58" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F58" s="7">
@@ -1845,15 +1920,15 @@
         <v>29.0</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E59" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E59" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F59" s="7">
@@ -1869,15 +1944,15 @@
         <v>30.0</v>
       </c>
       <c r="B60" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C60" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E60" s="13" t="s">
+      <c r="E60" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F60" s="7">
@@ -1893,15 +1968,15 @@
         <v>30.0</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E61" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E61" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F61" s="7">
@@ -1917,15 +1992,15 @@
         <v>31.0</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E62" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E62" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F62" s="7">
@@ -1941,15 +2016,15 @@
         <v>31.0</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E63" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E63" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F63" s="7">
@@ -1965,15 +2040,15 @@
         <v>32.0</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E64" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E64" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F64" s="7">
@@ -1989,15 +2064,15 @@
         <v>32.0</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E65" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E65" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F65" s="7">
@@ -2013,15 +2088,15 @@
         <v>33.0</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E66" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E66" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F66" s="7">
@@ -2037,15 +2112,15 @@
         <v>33.0</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E67" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E67" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F67" s="7">
@@ -2061,15 +2136,15 @@
         <v>34.0</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E68" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E68" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F68" s="7">
@@ -2085,15 +2160,15 @@
         <v>34.0</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E69" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E69" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F69" s="7">
@@ -2109,15 +2184,15 @@
         <v>35.0</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E70" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E70" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F70" s="7">
@@ -2133,15 +2208,15 @@
         <v>35.0</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E71" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E71" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F71" s="7">
@@ -2157,15 +2232,15 @@
         <v>36.0</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E72" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E72" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F72" s="7">
@@ -2181,15 +2256,15 @@
         <v>36.0</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E73" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E73" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F73" s="7">
@@ -2205,17 +2280,23 @@
         <v>37.0</v>
       </c>
       <c r="B74" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D74" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C74" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D74" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E74" s="10"/>
-      <c r="F74" s="11"/>
-      <c r="G74" s="11"/>
+      <c r="E74" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F74" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G74" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H74" s="8"/>
     </row>
     <row r="75" ht="22.5" customHeight="1">
@@ -2223,17 +2304,23 @@
         <v>37.0</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C75" s="14" t="s">
-        <v>24</v>
+        <v>16</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E75" s="10"/>
-      <c r="F75" s="11"/>
-      <c r="G75" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F75" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G75" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H75" s="8"/>
     </row>
     <row r="76" ht="22.5" customHeight="1">
@@ -2241,17 +2328,23 @@
         <v>38.0</v>
       </c>
       <c r="B76" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D76" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C76" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D76" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E76" s="10"/>
-      <c r="F76" s="11"/>
-      <c r="G76" s="11"/>
+      <c r="E76" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F76" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G76" s="7">
+        <v>46279.0</v>
+      </c>
       <c r="H76" s="8"/>
     </row>
     <row r="77" ht="22.5" customHeight="1">
@@ -2259,17 +2352,23 @@
         <v>38.0</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C77" s="14" t="s">
-        <v>24</v>
+        <v>16</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E77" s="10"/>
-      <c r="F77" s="11"/>
-      <c r="G77" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F77" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G77" s="7">
+        <v>46279.0</v>
+      </c>
       <c r="H77" s="8"/>
     </row>
     <row r="78" ht="22.5" customHeight="1">
@@ -2277,15 +2376,15 @@
         <v>39.0</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E78" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E78" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F78" s="7">
@@ -2301,15 +2400,15 @@
         <v>39.0</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E79" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E79" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F79" s="7">
@@ -2325,15 +2424,15 @@
         <v>40.0</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E80" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E80" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F80" s="7">
@@ -2349,15 +2448,15 @@
         <v>40.0</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E81" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E81" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F81" s="7">
@@ -2373,17 +2472,23 @@
         <v>41.0</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E82" s="10"/>
-      <c r="F82" s="11"/>
-      <c r="G82" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F82" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G82" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H82" s="8"/>
     </row>
     <row r="83" ht="22.5" customHeight="1">
@@ -2391,17 +2496,23 @@
         <v>41.0</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E83" s="10"/>
-      <c r="F83" s="11"/>
-      <c r="G83" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F83" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G83" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H83" s="8"/>
     </row>
     <row r="84" ht="22.5" customHeight="1">
@@ -2409,17 +2520,23 @@
         <v>42.0</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E84" s="10"/>
-      <c r="F84" s="11"/>
-      <c r="G84" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E84" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F84" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G84" s="7">
+        <v>46279.0</v>
+      </c>
       <c r="H84" s="8"/>
     </row>
     <row r="85" ht="22.5" customHeight="1">
@@ -2427,17 +2544,23 @@
         <v>42.0</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E85" s="10"/>
-      <c r="F85" s="11"/>
-      <c r="G85" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E85" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F85" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G85" s="7">
+        <v>46279.0</v>
+      </c>
       <c r="H85" s="8"/>
     </row>
     <row r="86" ht="22.5" customHeight="1">
@@ -2445,15 +2568,15 @@
         <v>43.0</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E86" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E86" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F86" s="7">
@@ -2469,15 +2592,15 @@
         <v>43.0</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E87" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E87" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F87" s="7">
@@ -2493,15 +2616,15 @@
         <v>44.0</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E88" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E88" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F88" s="7">
@@ -2517,15 +2640,15 @@
         <v>44.0</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E89" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E89" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F89" s="7">
@@ -2541,17 +2664,23 @@
         <v>45.0</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E90" s="10"/>
-      <c r="F90" s="11"/>
-      <c r="G90" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F90" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G90" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H90" s="8"/>
     </row>
     <row r="91" ht="22.5" customHeight="1">
@@ -2559,17 +2688,23 @@
         <v>45.0</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E91" s="10"/>
-      <c r="F91" s="11"/>
-      <c r="G91" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F91" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G91" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H91" s="8"/>
     </row>
     <row r="92" ht="22.5" customHeight="1">
@@ -2577,17 +2712,23 @@
         <v>46.0</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E92" s="10"/>
-      <c r="F92" s="11"/>
-      <c r="G92" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F92" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G92" s="7">
+        <v>46279.0</v>
+      </c>
       <c r="H92" s="8"/>
     </row>
     <row r="93" ht="22.5" customHeight="1">
@@ -2595,17 +2736,23 @@
         <v>46.0</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E93" s="10"/>
-      <c r="F93" s="11"/>
-      <c r="G93" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F93" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G93" s="7">
+        <v>46279.0</v>
+      </c>
       <c r="H93" s="8"/>
     </row>
     <row r="94" ht="22.5" customHeight="1">
@@ -2613,15 +2760,15 @@
         <v>47.0</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C94" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D94" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E94" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E94" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F94" s="7">
@@ -2637,15 +2784,15 @@
         <v>47.0</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E95" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E95" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F95" s="7">
@@ -2661,15 +2808,15 @@
         <v>48.0</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D96" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E96" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E96" s="16" t="s">
         <v>11</v>
       </c>
       <c r="F96" s="7">
@@ -2685,15 +2832,15 @@
         <v>48.0</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E97" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E97" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F97" s="7">
@@ -2709,17 +2856,23 @@
         <v>49.0</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C98" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="D98" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E98" s="10"/>
-      <c r="F98" s="11"/>
-      <c r="G98" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E98" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F98" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G98" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H98" s="8"/>
     </row>
     <row r="99" ht="22.5" customHeight="1">
@@ -2727,17 +2880,23 @@
         <v>49.0</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C99" s="14" t="s">
-        <v>24</v>
+        <v>16</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="D99" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E99" s="10"/>
-      <c r="F99" s="11"/>
-      <c r="G99" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" s="7">
+        <v>46249.0</v>
+      </c>
+      <c r="G99" s="7">
+        <v>46265.0</v>
+      </c>
       <c r="H99" s="8"/>
     </row>
     <row r="100" ht="22.5" customHeight="1">
@@ -2745,17 +2904,23 @@
         <v>50.0</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C100" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="D100" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E100" s="10"/>
-      <c r="F100" s="11"/>
-      <c r="G100" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="E100" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F100" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G100" s="7">
+        <v>46279.0</v>
+      </c>
       <c r="H100" s="8"/>
     </row>
     <row r="101" ht="22.5" customHeight="1">
@@ -2763,173 +2928,179 @@
         <v>50.0</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C101" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F101" s="7">
+        <v>46266.0</v>
+      </c>
+      <c r="G101" s="7">
+        <v>46279.0</v>
+      </c>
+      <c r="H101" s="8"/>
+    </row>
+    <row r="102" ht="22.5" customHeight="1">
+      <c r="A102" s="18"/>
+      <c r="B102" s="8"/>
+      <c r="C102" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D101" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E101" s="10"/>
-      <c r="F101" s="11"/>
-      <c r="G101" s="11"/>
-      <c r="H101" s="8"/>
-    </row>
-    <row r="102" ht="22.5" customHeight="1">
-      <c r="A102" s="17"/>
-      <c r="B102" s="8"/>
-      <c r="C102" s="14" t="s">
+      <c r="D102" s="8"/>
+      <c r="E102" s="19"/>
+      <c r="F102" s="14"/>
+      <c r="G102" s="14"/>
+      <c r="H102" s="8"/>
+    </row>
+    <row r="103" ht="22.5" customHeight="1">
+      <c r="A103" s="18"/>
+      <c r="B103" s="8"/>
+      <c r="C103" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D102" s="8"/>
-      <c r="E102" s="18"/>
-      <c r="F102" s="11"/>
-      <c r="G102" s="11"/>
-      <c r="H102" s="8"/>
-    </row>
-    <row r="103" ht="22.5" customHeight="1">
-      <c r="A103" s="17"/>
-      <c r="B103" s="8"/>
-      <c r="C103" s="14" t="s">
+      <c r="D103" s="8"/>
+      <c r="E103" s="19"/>
+      <c r="F103" s="14"/>
+      <c r="G103" s="14"/>
+      <c r="H103" s="8"/>
+    </row>
+    <row r="104" ht="22.5" customHeight="1">
+      <c r="A104" s="18"/>
+      <c r="B104" s="8"/>
+      <c r="C104" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D103" s="8"/>
-      <c r="E103" s="18"/>
-      <c r="F103" s="11"/>
-      <c r="G103" s="11"/>
-      <c r="H103" s="8"/>
-    </row>
-    <row r="104" ht="22.5" customHeight="1">
-      <c r="A104" s="17"/>
-      <c r="B104" s="8"/>
-      <c r="C104" s="14" t="s">
+      <c r="D104" s="8"/>
+      <c r="E104" s="19"/>
+      <c r="F104" s="14"/>
+      <c r="G104" s="14"/>
+      <c r="H104" s="8"/>
+    </row>
+    <row r="105" ht="22.5" customHeight="1">
+      <c r="A105" s="18"/>
+      <c r="B105" s="8"/>
+      <c r="C105" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D104" s="8"/>
-      <c r="E104" s="18"/>
-      <c r="F104" s="11"/>
-      <c r="G104" s="11"/>
-      <c r="H104" s="8"/>
-    </row>
-    <row r="105" ht="22.5" customHeight="1">
-      <c r="A105" s="17"/>
-      <c r="B105" s="8"/>
-      <c r="C105" s="14" t="s">
+      <c r="D105" s="8"/>
+      <c r="E105" s="19"/>
+      <c r="F105" s="14"/>
+      <c r="G105" s="14"/>
+      <c r="H105" s="8"/>
+    </row>
+    <row r="106" ht="22.5" customHeight="1">
+      <c r="A106" s="18"/>
+      <c r="B106" s="8"/>
+      <c r="C106" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D105" s="8"/>
-      <c r="E105" s="18"/>
-      <c r="F105" s="11"/>
-      <c r="G105" s="11"/>
-      <c r="H105" s="8"/>
-    </row>
-    <row r="106" ht="22.5" customHeight="1">
-      <c r="A106" s="17"/>
-      <c r="B106" s="8"/>
-      <c r="C106" s="14" t="s">
+      <c r="D106" s="8"/>
+      <c r="E106" s="19"/>
+      <c r="F106" s="14"/>
+      <c r="G106" s="14"/>
+      <c r="H106" s="8"/>
+    </row>
+    <row r="107" ht="22.5" customHeight="1">
+      <c r="A107" s="18"/>
+      <c r="B107" s="8"/>
+      <c r="C107" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D106" s="8"/>
-      <c r="E106" s="18"/>
-      <c r="F106" s="11"/>
-      <c r="G106" s="11"/>
-      <c r="H106" s="8"/>
-    </row>
-    <row r="107" ht="22.5" customHeight="1">
-      <c r="A107" s="17"/>
-      <c r="B107" s="8"/>
-      <c r="C107" s="14" t="s">
+      <c r="D107" s="8"/>
+      <c r="E107" s="19"/>
+      <c r="F107" s="14"/>
+      <c r="G107" s="14"/>
+      <c r="H107" s="8"/>
+    </row>
+    <row r="108" ht="22.5" customHeight="1">
+      <c r="A108" s="18"/>
+      <c r="B108" s="8"/>
+      <c r="C108" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D107" s="8"/>
-      <c r="E107" s="18"/>
-      <c r="F107" s="11"/>
-      <c r="G107" s="11"/>
-      <c r="H107" s="8"/>
-    </row>
-    <row r="108" ht="22.5" customHeight="1">
-      <c r="A108" s="17"/>
-      <c r="B108" s="8"/>
-      <c r="C108" s="14" t="s">
+      <c r="D108" s="8"/>
+      <c r="E108" s="19"/>
+      <c r="F108" s="14"/>
+      <c r="G108" s="14"/>
+      <c r="H108" s="8"/>
+    </row>
+    <row r="109" ht="22.5" customHeight="1">
+      <c r="A109" s="18"/>
+      <c r="B109" s="8"/>
+      <c r="C109" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D108" s="8"/>
-      <c r="E108" s="18"/>
-      <c r="F108" s="11"/>
-      <c r="G108" s="11"/>
-      <c r="H108" s="8"/>
-    </row>
-    <row r="109" ht="22.5" customHeight="1">
-      <c r="A109" s="17"/>
-      <c r="B109" s="8"/>
-      <c r="C109" s="14" t="s">
+      <c r="D109" s="8"/>
+      <c r="E109" s="19"/>
+      <c r="F109" s="14"/>
+      <c r="G109" s="14"/>
+      <c r="H109" s="8"/>
+    </row>
+    <row r="110" ht="22.5" customHeight="1">
+      <c r="A110" s="18"/>
+      <c r="B110" s="8"/>
+      <c r="C110" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D109" s="8"/>
-      <c r="E109" s="18"/>
-      <c r="F109" s="11"/>
-      <c r="G109" s="11"/>
-      <c r="H109" s="8"/>
-    </row>
-    <row r="110" ht="22.5" customHeight="1">
-      <c r="A110" s="17"/>
-      <c r="B110" s="8"/>
-      <c r="C110" s="14" t="s">
+      <c r="D110" s="8"/>
+      <c r="E110" s="19"/>
+      <c r="F110" s="14"/>
+      <c r="G110" s="14"/>
+      <c r="H110" s="8"/>
+    </row>
+    <row r="111" ht="22.5" customHeight="1">
+      <c r="A111" s="18"/>
+      <c r="B111" s="8"/>
+      <c r="C111" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D110" s="8"/>
-      <c r="E110" s="18"/>
-      <c r="F110" s="11"/>
-      <c r="G110" s="11"/>
-      <c r="H110" s="8"/>
-    </row>
-    <row r="111" ht="22.5" customHeight="1">
-      <c r="A111" s="17"/>
-      <c r="B111" s="8"/>
-      <c r="C111" s="14" t="s">
+      <c r="D111" s="8"/>
+      <c r="E111" s="19"/>
+      <c r="F111" s="14"/>
+      <c r="G111" s="14"/>
+      <c r="H111" s="8"/>
+    </row>
+    <row r="112" ht="22.5" customHeight="1">
+      <c r="A112" s="18"/>
+      <c r="B112" s="8"/>
+      <c r="C112" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D111" s="8"/>
-      <c r="E111" s="18"/>
-      <c r="F111" s="11"/>
-      <c r="G111" s="11"/>
-      <c r="H111" s="8"/>
-    </row>
-    <row r="112" ht="22.5" customHeight="1">
-      <c r="A112" s="17"/>
-      <c r="B112" s="8"/>
-      <c r="C112" s="14" t="s">
+      <c r="D112" s="8"/>
+      <c r="E112" s="19"/>
+      <c r="F112" s="14"/>
+      <c r="G112" s="14"/>
+      <c r="H112" s="8"/>
+    </row>
+    <row r="113" ht="22.5" customHeight="1">
+      <c r="A113" s="18"/>
+      <c r="B113" s="8"/>
+      <c r="C113" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D112" s="8"/>
-      <c r="E112" s="18"/>
-      <c r="F112" s="11"/>
-      <c r="G112" s="11"/>
-      <c r="H112" s="8"/>
-    </row>
-    <row r="113" ht="22.5" customHeight="1">
-      <c r="A113" s="17"/>
-      <c r="B113" s="8"/>
-      <c r="C113" s="14" t="s">
+      <c r="D113" s="8"/>
+      <c r="E113" s="19"/>
+      <c r="F113" s="14"/>
+      <c r="G113" s="14"/>
+      <c r="H113" s="8"/>
+    </row>
+    <row r="114" ht="22.5" customHeight="1">
+      <c r="A114" s="18"/>
+      <c r="B114" s="8"/>
+      <c r="C114" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D113" s="8"/>
-      <c r="E113" s="18"/>
-      <c r="F113" s="11"/>
-      <c r="G113" s="11"/>
-      <c r="H113" s="8"/>
-    </row>
-    <row r="114" ht="22.5" customHeight="1">
-      <c r="A114" s="17"/>
-      <c r="B114" s="8"/>
-      <c r="C114" s="14" t="s">
-        <v>24</v>
-      </c>
       <c r="D114" s="8"/>
-      <c r="E114" s="18"/>
-      <c r="F114" s="11"/>
-      <c r="G114" s="11"/>
+      <c r="E114" s="19"/>
+      <c r="F114" s="14"/>
+      <c r="G114" s="14"/>
       <c r="H114" s="8"/>
     </row>
   </sheetData>
@@ -2944,155 +3115,170 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="D2"/>
-    <hyperlink r:id="rId2" ref="D3"/>
-    <hyperlink r:id="rId3" ref="D4"/>
-    <hyperlink r:id="rId4" ref="D5"/>
-    <hyperlink r:id="rId5" ref="D6"/>
-    <hyperlink r:id="rId6" ref="D7"/>
-    <hyperlink r:id="rId7" ref="D8"/>
-    <hyperlink r:id="rId8" ref="D9"/>
-    <hyperlink r:id="rId9" ref="D10"/>
-    <hyperlink r:id="rId10" ref="D11"/>
-    <hyperlink r:id="rId11" ref="D12"/>
-    <hyperlink r:id="rId12" ref="D13"/>
-    <hyperlink r:id="rId13" ref="D14"/>
-    <hyperlink r:id="rId14" ref="D15"/>
-    <hyperlink r:id="rId15" ref="D16"/>
-    <hyperlink r:id="rId16" ref="D17"/>
-    <hyperlink r:id="rId17" ref="D18"/>
-    <hyperlink r:id="rId18" ref="E18"/>
-    <hyperlink r:id="rId19" ref="D19"/>
-    <hyperlink r:id="rId20" ref="E19"/>
-    <hyperlink r:id="rId21" ref="D20"/>
-    <hyperlink r:id="rId22" ref="E20"/>
-    <hyperlink r:id="rId23" ref="D21"/>
-    <hyperlink r:id="rId24" ref="E21"/>
-    <hyperlink r:id="rId25" ref="D22"/>
-    <hyperlink r:id="rId26" ref="E22"/>
-    <hyperlink r:id="rId27" ref="D23"/>
-    <hyperlink r:id="rId28" ref="E23"/>
-    <hyperlink r:id="rId29" ref="D24"/>
-    <hyperlink r:id="rId30" ref="E24"/>
-    <hyperlink r:id="rId31" ref="D25"/>
-    <hyperlink r:id="rId32" ref="E25"/>
-    <hyperlink r:id="rId33" ref="D26"/>
-    <hyperlink r:id="rId34" ref="D27"/>
-    <hyperlink r:id="rId35" ref="D28"/>
-    <hyperlink r:id="rId36" ref="D29"/>
-    <hyperlink r:id="rId37" ref="D30"/>
-    <hyperlink r:id="rId38" ref="E30"/>
-    <hyperlink r:id="rId39" ref="D31"/>
-    <hyperlink r:id="rId40" ref="E31"/>
-    <hyperlink r:id="rId41" ref="D32"/>
-    <hyperlink r:id="rId42" ref="E32"/>
-    <hyperlink r:id="rId43" ref="D33"/>
-    <hyperlink r:id="rId44" ref="E33"/>
-    <hyperlink r:id="rId45" ref="D34"/>
-    <hyperlink r:id="rId46" ref="E34"/>
-    <hyperlink r:id="rId47" ref="D35"/>
-    <hyperlink r:id="rId48" ref="E35"/>
-    <hyperlink r:id="rId49" ref="D36"/>
-    <hyperlink r:id="rId50" ref="E36"/>
-    <hyperlink r:id="rId51" ref="D37"/>
-    <hyperlink r:id="rId52" ref="E37"/>
-    <hyperlink r:id="rId53" ref="D38"/>
-    <hyperlink r:id="rId54" ref="E38"/>
+    <hyperlink r:id="rId2" location="gid=353009147" ref="E2"/>
+    <hyperlink r:id="rId3" ref="D3"/>
+    <hyperlink r:id="rId4" ref="D4"/>
+    <hyperlink r:id="rId5" location="gid=403914780" ref="E4"/>
+    <hyperlink r:id="rId6" ref="D5"/>
+    <hyperlink r:id="rId7" ref="D6"/>
+    <hyperlink r:id="rId8" location="gid=1115831507" ref="E6"/>
+    <hyperlink r:id="rId9" ref="D7"/>
+    <hyperlink r:id="rId10" ref="D8"/>
+    <hyperlink r:id="rId11" ref="D9"/>
+    <hyperlink r:id="rId12" ref="D10"/>
+    <hyperlink r:id="rId13" ref="D11"/>
+    <hyperlink r:id="rId14" ref="D12"/>
+    <hyperlink r:id="rId15" ref="D13"/>
+    <hyperlink r:id="rId16" ref="D14"/>
+    <hyperlink r:id="rId17" ref="D15"/>
+    <hyperlink r:id="rId18" ref="D16"/>
+    <hyperlink r:id="rId19" ref="D17"/>
+    <hyperlink r:id="rId20" ref="D18"/>
+    <hyperlink r:id="rId21" ref="E18"/>
+    <hyperlink r:id="rId22" ref="D19"/>
+    <hyperlink r:id="rId23" ref="E19"/>
+    <hyperlink r:id="rId24" ref="D20"/>
+    <hyperlink r:id="rId25" ref="E20"/>
+    <hyperlink r:id="rId26" ref="D21"/>
+    <hyperlink r:id="rId27" ref="E21"/>
+    <hyperlink r:id="rId28" ref="D22"/>
+    <hyperlink r:id="rId29" ref="E22"/>
+    <hyperlink r:id="rId30" ref="D23"/>
+    <hyperlink r:id="rId31" ref="E23"/>
+    <hyperlink r:id="rId32" ref="D24"/>
+    <hyperlink r:id="rId33" ref="E24"/>
+    <hyperlink r:id="rId34" ref="D25"/>
+    <hyperlink r:id="rId35" ref="E25"/>
+    <hyperlink r:id="rId36" ref="D26"/>
+    <hyperlink r:id="rId37" ref="D28"/>
+    <hyperlink r:id="rId38" ref="D30"/>
+    <hyperlink r:id="rId39" ref="E30"/>
+    <hyperlink r:id="rId40" ref="D31"/>
+    <hyperlink r:id="rId41" ref="E31"/>
+    <hyperlink r:id="rId42" ref="D32"/>
+    <hyperlink r:id="rId43" ref="E32"/>
+    <hyperlink r:id="rId44" ref="D33"/>
+    <hyperlink r:id="rId45" ref="E33"/>
+    <hyperlink r:id="rId46" ref="D34"/>
+    <hyperlink r:id="rId47" ref="E34"/>
+    <hyperlink r:id="rId48" ref="D35"/>
+    <hyperlink r:id="rId49" ref="E35"/>
+    <hyperlink r:id="rId50" ref="D36"/>
+    <hyperlink r:id="rId51" ref="E36"/>
+    <hyperlink r:id="rId52" ref="D37"/>
+    <hyperlink r:id="rId53" ref="E37"/>
+    <hyperlink r:id="rId54" ref="D38"/>
     <hyperlink r:id="rId55" ref="D39"/>
-    <hyperlink r:id="rId56" ref="E39"/>
-    <hyperlink r:id="rId57" ref="D40"/>
-    <hyperlink r:id="rId58" ref="D41"/>
-    <hyperlink r:id="rId59" ref="D42"/>
-    <hyperlink r:id="rId60" ref="D43"/>
-    <hyperlink r:id="rId61" ref="D44"/>
-    <hyperlink r:id="rId62" ref="D45"/>
-    <hyperlink r:id="rId63" ref="D46"/>
-    <hyperlink r:id="rId64" ref="D47"/>
-    <hyperlink r:id="rId65" ref="D48"/>
-    <hyperlink r:id="rId66" ref="D49"/>
-    <hyperlink r:id="rId67" ref="D50"/>
-    <hyperlink r:id="rId68" ref="D51"/>
-    <hyperlink r:id="rId69" ref="D52"/>
-    <hyperlink r:id="rId70" ref="D53"/>
-    <hyperlink r:id="rId71" ref="D54"/>
-    <hyperlink r:id="rId72" ref="D55"/>
-    <hyperlink r:id="rId73" ref="D56"/>
-    <hyperlink r:id="rId74" ref="D57"/>
-    <hyperlink r:id="rId75" ref="D58"/>
-    <hyperlink r:id="rId76" ref="E58"/>
-    <hyperlink r:id="rId77" ref="D59"/>
-    <hyperlink r:id="rId78" ref="E59"/>
-    <hyperlink r:id="rId79" ref="D60"/>
-    <hyperlink r:id="rId80" ref="E60"/>
-    <hyperlink r:id="rId81" ref="D61"/>
-    <hyperlink r:id="rId82" ref="E61"/>
-    <hyperlink r:id="rId83" ref="D62"/>
-    <hyperlink r:id="rId84" ref="E62"/>
-    <hyperlink r:id="rId85" ref="D63"/>
-    <hyperlink r:id="rId86" ref="E63"/>
-    <hyperlink r:id="rId87" ref="D64"/>
-    <hyperlink r:id="rId88" ref="E64"/>
-    <hyperlink r:id="rId89" ref="D65"/>
-    <hyperlink r:id="rId90" ref="E65"/>
-    <hyperlink r:id="rId91" ref="D66"/>
-    <hyperlink r:id="rId92" ref="E66"/>
-    <hyperlink r:id="rId93" ref="D67"/>
-    <hyperlink r:id="rId94" ref="E67"/>
-    <hyperlink r:id="rId95" ref="D68"/>
-    <hyperlink r:id="rId96" ref="E68"/>
-    <hyperlink r:id="rId97" ref="D69"/>
-    <hyperlink r:id="rId98" ref="E69"/>
-    <hyperlink r:id="rId99" ref="D70"/>
-    <hyperlink r:id="rId100" ref="E70"/>
-    <hyperlink r:id="rId101" ref="D71"/>
-    <hyperlink r:id="rId102" ref="E71"/>
-    <hyperlink r:id="rId103" ref="D72"/>
-    <hyperlink r:id="rId104" ref="E72"/>
-    <hyperlink r:id="rId105" ref="D73"/>
-    <hyperlink r:id="rId106" ref="E73"/>
-    <hyperlink r:id="rId107" ref="D74"/>
+    <hyperlink r:id="rId56" ref="D40"/>
+    <hyperlink r:id="rId57" ref="D41"/>
+    <hyperlink r:id="rId58" ref="D42"/>
+    <hyperlink r:id="rId59" ref="D43"/>
+    <hyperlink r:id="rId60" ref="D44"/>
+    <hyperlink r:id="rId61" ref="D45"/>
+    <hyperlink r:id="rId62" ref="D46"/>
+    <hyperlink r:id="rId63" ref="D47"/>
+    <hyperlink r:id="rId64" ref="D48"/>
+    <hyperlink r:id="rId65" ref="D49"/>
+    <hyperlink r:id="rId66" ref="D50"/>
+    <hyperlink r:id="rId67" ref="D51"/>
+    <hyperlink r:id="rId68" ref="D52"/>
+    <hyperlink r:id="rId69" ref="D53"/>
+    <hyperlink r:id="rId70" ref="D54"/>
+    <hyperlink r:id="rId71" ref="D55"/>
+    <hyperlink r:id="rId72" ref="D56"/>
+    <hyperlink r:id="rId73" ref="D57"/>
+    <hyperlink r:id="rId74" ref="D58"/>
+    <hyperlink r:id="rId75" ref="E58"/>
+    <hyperlink r:id="rId76" ref="D59"/>
+    <hyperlink r:id="rId77" ref="E59"/>
+    <hyperlink r:id="rId78" ref="D60"/>
+    <hyperlink r:id="rId79" ref="E60"/>
+    <hyperlink r:id="rId80" ref="D61"/>
+    <hyperlink r:id="rId81" ref="E61"/>
+    <hyperlink r:id="rId82" ref="D62"/>
+    <hyperlink r:id="rId83" ref="E62"/>
+    <hyperlink r:id="rId84" ref="D63"/>
+    <hyperlink r:id="rId85" ref="E63"/>
+    <hyperlink r:id="rId86" ref="D64"/>
+    <hyperlink r:id="rId87" ref="E64"/>
+    <hyperlink r:id="rId88" ref="D65"/>
+    <hyperlink r:id="rId89" ref="E65"/>
+    <hyperlink r:id="rId90" ref="D66"/>
+    <hyperlink r:id="rId91" ref="E66"/>
+    <hyperlink r:id="rId92" ref="D67"/>
+    <hyperlink r:id="rId93" ref="E67"/>
+    <hyperlink r:id="rId94" ref="D68"/>
+    <hyperlink r:id="rId95" ref="E68"/>
+    <hyperlink r:id="rId96" ref="D69"/>
+    <hyperlink r:id="rId97" ref="E69"/>
+    <hyperlink r:id="rId98" ref="D70"/>
+    <hyperlink r:id="rId99" ref="E70"/>
+    <hyperlink r:id="rId100" ref="D71"/>
+    <hyperlink r:id="rId101" ref="E71"/>
+    <hyperlink r:id="rId102" ref="D72"/>
+    <hyperlink r:id="rId103" ref="E72"/>
+    <hyperlink r:id="rId104" ref="D73"/>
+    <hyperlink r:id="rId105" ref="E73"/>
+    <hyperlink r:id="rId106" ref="D74"/>
+    <hyperlink r:id="rId107" location="gid=814312368" ref="E74"/>
     <hyperlink r:id="rId108" ref="D75"/>
-    <hyperlink r:id="rId109" ref="D76"/>
-    <hyperlink r:id="rId110" ref="D77"/>
-    <hyperlink r:id="rId111" ref="D78"/>
-    <hyperlink r:id="rId112" ref="E78"/>
-    <hyperlink r:id="rId113" ref="D79"/>
-    <hyperlink r:id="rId114" ref="E79"/>
-    <hyperlink r:id="rId115" ref="D80"/>
-    <hyperlink r:id="rId116" ref="E80"/>
-    <hyperlink r:id="rId117" ref="D81"/>
-    <hyperlink r:id="rId118" ref="E81"/>
-    <hyperlink r:id="rId119" ref="D82"/>
-    <hyperlink r:id="rId120" ref="D83"/>
-    <hyperlink r:id="rId121" ref="D84"/>
-    <hyperlink r:id="rId122" ref="D85"/>
-    <hyperlink r:id="rId123" ref="D86"/>
-    <hyperlink r:id="rId124" ref="E86"/>
-    <hyperlink r:id="rId125" ref="D87"/>
-    <hyperlink r:id="rId126" ref="E87"/>
-    <hyperlink r:id="rId127" ref="D88"/>
-    <hyperlink r:id="rId128" ref="E88"/>
-    <hyperlink r:id="rId129" ref="D89"/>
-    <hyperlink r:id="rId130" ref="E89"/>
-    <hyperlink r:id="rId131" ref="D90"/>
-    <hyperlink r:id="rId132" ref="D91"/>
-    <hyperlink r:id="rId133" ref="D92"/>
-    <hyperlink r:id="rId134" ref="D93"/>
-    <hyperlink r:id="rId135" ref="D94"/>
-    <hyperlink r:id="rId136" ref="E94"/>
-    <hyperlink r:id="rId137" ref="D95"/>
-    <hyperlink r:id="rId138" ref="E95"/>
-    <hyperlink r:id="rId139" ref="D96"/>
-    <hyperlink r:id="rId140" ref="E96"/>
-    <hyperlink r:id="rId141" ref="D97"/>
-    <hyperlink r:id="rId142" ref="E97"/>
-    <hyperlink r:id="rId143" ref="D98"/>
-    <hyperlink r:id="rId144" ref="D99"/>
-    <hyperlink r:id="rId145" ref="D100"/>
-    <hyperlink r:id="rId146" ref="D101"/>
+    <hyperlink r:id="rId109" location="gid=1724619799" ref="E75"/>
+    <hyperlink r:id="rId110" ref="D76"/>
+    <hyperlink r:id="rId111" location="gid=783188431" ref="E76"/>
+    <hyperlink r:id="rId112" ref="D77"/>
+    <hyperlink r:id="rId113" location="gid=1517587847" ref="E77"/>
+    <hyperlink r:id="rId114" ref="D78"/>
+    <hyperlink r:id="rId115" ref="E78"/>
+    <hyperlink r:id="rId116" ref="D79"/>
+    <hyperlink r:id="rId117" ref="E79"/>
+    <hyperlink r:id="rId118" ref="D80"/>
+    <hyperlink r:id="rId119" ref="E80"/>
+    <hyperlink r:id="rId120" ref="D81"/>
+    <hyperlink r:id="rId121" ref="E81"/>
+    <hyperlink r:id="rId122" ref="D82"/>
+    <hyperlink r:id="rId123" location="gid=2081753222" ref="E82"/>
+    <hyperlink r:id="rId124" ref="D83"/>
+    <hyperlink r:id="rId125" location="gid=2058403121" ref="E83"/>
+    <hyperlink r:id="rId126" ref="D84"/>
+    <hyperlink r:id="rId127" location="gid=430859523" ref="E84"/>
+    <hyperlink r:id="rId128" ref="D85"/>
+    <hyperlink r:id="rId129" location="gid=1686693134" ref="E85"/>
+    <hyperlink r:id="rId130" ref="D86"/>
+    <hyperlink r:id="rId131" ref="E86"/>
+    <hyperlink r:id="rId132" ref="D87"/>
+    <hyperlink r:id="rId133" ref="E87"/>
+    <hyperlink r:id="rId134" ref="D88"/>
+    <hyperlink r:id="rId135" ref="E88"/>
+    <hyperlink r:id="rId136" ref="D89"/>
+    <hyperlink r:id="rId137" ref="E89"/>
+    <hyperlink r:id="rId138" ref="D90"/>
+    <hyperlink r:id="rId139" location="gid=1542557206" ref="E90"/>
+    <hyperlink r:id="rId140" ref="D91"/>
+    <hyperlink r:id="rId141" location="gid=176968273" ref="E91"/>
+    <hyperlink r:id="rId142" ref="D92"/>
+    <hyperlink r:id="rId143" location="gid=1542557206" ref="E92"/>
+    <hyperlink r:id="rId144" ref="D93"/>
+    <hyperlink r:id="rId145" location="gid=736062176" ref="E93"/>
+    <hyperlink r:id="rId146" ref="D94"/>
+    <hyperlink r:id="rId147" ref="E94"/>
+    <hyperlink r:id="rId148" ref="D95"/>
+    <hyperlink r:id="rId149" ref="E95"/>
+    <hyperlink r:id="rId150" ref="D96"/>
+    <hyperlink r:id="rId151" ref="E96"/>
+    <hyperlink r:id="rId152" ref="D97"/>
+    <hyperlink r:id="rId153" ref="E97"/>
+    <hyperlink r:id="rId154" ref="D98"/>
+    <hyperlink r:id="rId155" location="gid=716172970" ref="E98"/>
+    <hyperlink r:id="rId156" ref="D99"/>
+    <hyperlink r:id="rId157" location="gid=1974051076" ref="E99"/>
+    <hyperlink r:id="rId158" ref="D100"/>
+    <hyperlink r:id="rId159" location="gid=1321666791" ref="E100"/>
+    <hyperlink r:id="rId160" ref="D101"/>
+    <hyperlink r:id="rId161" location="gid=2103556022" ref="E101"/>
   </hyperlinks>
-  <drawing r:id="rId147"/>
+  <drawing r:id="rId162"/>
   <tableParts count="1">
-    <tablePart r:id="rId149"/>
+    <tablePart r:id="rId164"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>